<commit_message>
The real roster and the Denver game go live
- data/roster.xlsx is the team's 14-man roster, numbered 1-14; the names match
  the card profiles exactly, so this season's stats attach to the cards.
- games/ carries one game: vs Denver, 22 Aug 2026, 39-40. Exported by the
  previous build (no Minutes or Empty Net columns) — the importer reads by
  header name, so it loads clean and those columns read zero.
- A field player who covered a few shots in goal keeps a field player's card:
  the CARD's own position decides which stat strip and which overall it gets,
  not "did they face a shot". In this game a centre back faced one shot and
  would otherwise have been shown as a 100% keeper.
- The hosted roster assertion now compares against the committed file instead
  of a count typed into the probe, which had already gone stale (12 vs 14).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/roster.xlsx
+++ b/data/roster.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -424,212 +424,246 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v/>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Jack</v>
+        <v>C1C Jack P. Tierney</v>
       </c>
       <c r="C2" t="str">
         <v>CB</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>2027</v>
       </c>
       <c r="E2" t="str">
         <v>Y</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v/>
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>RJ</v>
+        <v>C1C Logan T Cook</v>
       </c>
       <c r="C3" t="str">
+        <v>CB</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2027</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>C1C Ryan S. Sansano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>LW</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2027</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>C1C Zachary D. Crane</v>
+      </c>
+      <c r="C5" t="str">
+        <v>GK</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2027</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>C1C Robert W. Garrett IV</v>
+      </c>
+      <c r="C6" t="str">
         <v>LB</v>
       </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v/>
-      </c>
-      <c r="B4" t="str">
-        <v>Ryan</v>
-      </c>
-      <c r="C4" t="str">
+      <c r="D6" t="str">
+        <v>2027</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>C1C Troy E. Miller</v>
+      </c>
+      <c r="C7" t="str">
         <v>RW</v>
       </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v/>
-      </c>
-      <c r="B5" t="str">
-        <v>Roman</v>
-      </c>
-      <c r="C5" t="str">
+      <c r="D7" t="str">
+        <v>2027</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>C2C Darian K. Presley</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CB</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2028</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>C2C Roman E. Trice</v>
+      </c>
+      <c r="C9" t="str">
         <v>P</v>
       </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v/>
-      </c>
-      <c r="B6" t="str">
-        <v>Charlie</v>
-      </c>
-      <c r="C6" t="str">
-        <v>LW</v>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <v>Evan</v>
-      </c>
-      <c r="C7" t="str">
-        <v>RB</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v/>
-      </c>
-      <c r="B8" t="str">
-        <v>Barrett</v>
-      </c>
-      <c r="C8" t="str">
-        <v>LB</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v/>
-      </c>
-      <c r="B9" t="str">
-        <v>Sean</v>
-      </c>
-      <c r="C9" t="str">
-        <v>LW</v>
-      </c>
       <c r="D9" t="str">
-        <v/>
+        <v>2028</v>
       </c>
       <c r="E9" t="str">
         <v>Y</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
-        <v/>
+      <c r="A10">
+        <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Christian</v>
+        <v>C3C Ian P. Cavendish</v>
       </c>
       <c r="C10" t="str">
-        <v>RW</v>
+        <v>CB</v>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>2029</v>
       </c>
       <c r="E10" t="str">
         <v>Y</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
-        <v/>
+      <c r="A11">
+        <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Ben</v>
+        <v>C3C Evan M. Feller</v>
       </c>
       <c r="C11" t="str">
+        <v>CB</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2029</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>C3C Tyler J. Ferguson</v>
+      </c>
+      <c r="C12" t="str">
         <v>P</v>
       </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v>Y</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v>Corn</v>
-      </c>
-      <c r="C12" t="str">
-        <v>GK</v>
-      </c>
       <c r="D12" t="str">
-        <v/>
+        <v>2029</v>
       </c>
       <c r="E12" t="str">
         <v>Y</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
-        <v/>
+      <c r="A13">
+        <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>Crane</v>
+        <v>C3C Charles B. Forth</v>
       </c>
       <c r="C13" t="str">
-        <v>GK</v>
+        <v>CB</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>2029</v>
       </c>
       <c r="E13" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>C3C Barrett S. Waldvogel</v>
+      </c>
+      <c r="C14" t="str">
+        <v>CB</v>
+      </c>
+      <c r="D14" t="str">
+        <v>2029</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>C3C Sean W. Windell</v>
+      </c>
+      <c r="C15" t="str">
+        <v>CB</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2029</v>
+      </c>
+      <c r="E15" t="str">
         <v>Y</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Listanowsky joins the stat roster as #15
Number counts up from the last used, position (LB) taken from his card, class
year from the cadet rank. A first-time device now starts with 15 players and
his card will carry a stat strip once he plays.

C2C Riley W. Lanham is still card-only.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/roster.xlsx
+++ b/data/roster.xlsx
@@ -397,10 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
     <col min="3" max="3" width="6.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" customWidth="1"/>
@@ -661,9 +661,26 @@
         <v>Y</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>C3C Henry J. Listanowsky</v>
+      </c>
+      <c r="C16" t="str">
+        <v>LB</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2029</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Y</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lanham joins the stat roster as #16 — roster and cards now agree
Position P from his card's "Circle", class year from the cadet rank, number
counting up. Every card-holding player is now on the stat roster: 16 players
on both sides, 3 coaches card-only as they should be.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/roster.xlsx
+++ b/data/roster.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -678,9 +678,26 @@
         <v>Y</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>C2C Riley W. Lanham</v>
+      </c>
+      <c r="C17" t="str">
+        <v>P</v>
+      </c>
+      <c r="D17" t="str">
+        <v>2028</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Y</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Forth is Right Wing and Waldvogel is Left Back — the bios were right
Owner confirmed the positions sent with the bios were the accurate ones, so
both files move together: the cards read Right Wing and Left Back, and
data/roster.xlsx reads RW and LB. This reverses the earlier sync, which had
made the cards follow the roster on the assumption the roster was authoritative.

Checked across the whole squad afterwards: no card and roster position
disagree.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/roster.xlsx
+++ b/data/roster.xlsx
@@ -618,7 +618,7 @@
         <v>C3C Charles B. Forth</v>
       </c>
       <c r="C13" t="str">
-        <v>CB</v>
+        <v>RW</v>
       </c>
       <c r="D13" t="str">
         <v>2029</v>
@@ -635,7 +635,7 @@
         <v>C3C Barrett S. Waldvogel</v>
       </c>
       <c r="C14" t="str">
-        <v>CB</v>
+        <v>LB</v>
       </c>
       <c r="D14" t="str">
         <v>2029</v>

</xml_diff>